<commit_message>
add onco/TS miR annotation to TableS3
</commit_message>
<xml_diff>
--- a/tables/TableS3.xlsx
+++ b/tables/TableS3.xlsx
@@ -107,6 +107,11 @@
           <t xml:space="preserve">Annotated-correlation</t>
         </is>
       </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OncomiR/TS miRNA</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -174,6 +179,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -269,6 +279,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -336,6 +351,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -403,6 +423,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -470,6 +495,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -537,6 +567,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -604,6 +639,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -671,6 +711,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -738,6 +783,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -805,6 +855,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -900,6 +955,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -995,6 +1055,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1062,6 +1127,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1129,6 +1199,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1196,6 +1271,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1263,6 +1343,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1330,6 +1415,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1397,6 +1487,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1464,6 +1559,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1531,6 +1631,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1598,6 +1703,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1665,6 +1775,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tumor suppressor</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1732,6 +1847,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1799,6 +1919,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tumor suppressor</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1866,6 +1991,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1933,6 +2063,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2000,6 +2135,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2067,6 +2207,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2134,6 +2279,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2201,6 +2351,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2268,6 +2423,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2335,6 +2495,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2402,6 +2567,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2469,6 +2639,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2536,6 +2711,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tumor suppressor</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2603,6 +2783,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2670,6 +2855,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tumor suppressor</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2737,6 +2927,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2804,6 +2999,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2871,6 +3071,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2938,6 +3143,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3005,6 +3215,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3072,6 +3287,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3167,6 +3387,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3234,6 +3459,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3301,6 +3531,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3368,6 +3603,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3435,6 +3675,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3502,6 +3747,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3569,6 +3819,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3636,6 +3891,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3703,6 +3963,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3770,6 +4035,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3837,6 +4107,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3904,6 +4179,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tumor suppressor</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3971,6 +4251,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tumor suppressor</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4038,6 +4323,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -4105,6 +4395,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tumor suppressor</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -4172,6 +4467,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -4239,6 +4539,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -4306,6 +4611,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4373,6 +4683,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OncomiR</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -4440,6 +4755,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OncomiR</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -4535,6 +4855,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -4602,6 +4927,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -4669,6 +4999,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -4736,6 +5071,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -4831,6 +5171,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -4898,6 +5243,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -4965,6 +5315,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -5032,6 +5387,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -5099,6 +5459,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -5166,6 +5531,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -5233,6 +5603,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -5300,6 +5675,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -5367,6 +5747,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -5434,6 +5819,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -5501,6 +5891,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -5568,6 +5963,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -5635,6 +6035,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tumor suppressor</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -5702,6 +6107,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -5769,6 +6179,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -5836,6 +6251,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -5903,6 +6323,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -5970,6 +6395,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OncomiR</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -6037,6 +6467,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -6104,6 +6539,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OncomiR</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -6171,6 +6611,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -6238,6 +6683,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -6305,6 +6755,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -6372,6 +6827,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -6439,6 +6899,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -6506,6 +6971,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -6573,6 +7043,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -6640,6 +7115,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -6707,6 +7187,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -6774,6 +7259,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -6841,6 +7331,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -6908,6 +7403,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -6975,6 +7475,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -7042,6 +7547,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -7109,6 +7619,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -7176,6 +7691,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -7243,6 +7763,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -7310,6 +7835,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -7377,6 +7907,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -7444,6 +7979,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -7511,6 +8051,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -7578,6 +8123,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OncomiR</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -7645,6 +8195,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -7712,6 +8267,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -7779,6 +8339,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -7846,6 +8411,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -7913,6 +8483,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -7980,6 +8555,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -8047,6 +8627,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -8114,6 +8699,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -8181,6 +8771,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -8248,6 +8843,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -8315,6 +8915,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -8382,6 +8987,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OncomiR</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -8449,6 +9059,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -8516,6 +9131,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -8583,6 +9203,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -8650,6 +9275,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -8717,6 +9347,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -8784,6 +9419,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -8851,6 +9491,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -8918,6 +9563,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -8985,6 +9635,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -9052,6 +9707,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -9119,6 +9779,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -9186,6 +9851,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -9253,6 +9923,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tumor suppressor</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -9320,6 +9995,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -9387,6 +10067,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -9454,6 +10139,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tumor suppressor</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -9521,6 +10211,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -9588,6 +10283,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -9655,6 +10355,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -9722,6 +10427,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -9789,6 +10499,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -9856,6 +10571,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T144" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -9923,6 +10643,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T145" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -9990,6 +10715,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T146" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OncomiR</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -10057,6 +10787,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T147" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OncomiR</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -10124,6 +10859,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T148" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -10191,6 +10931,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T149" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -10258,6 +11003,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T150" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OncomiR</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -10325,6 +11075,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T151" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OncomiR</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -10392,6 +11147,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OncomiR</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -10459,6 +11219,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T153" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OncomiR</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -10526,6 +11291,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -10593,6 +11363,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T155" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -10660,6 +11435,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T156" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OncomiR</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -10727,6 +11507,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T157" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -10794,6 +11579,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T158" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -10861,6 +11651,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T159" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -10928,6 +11723,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -10995,6 +11795,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T161" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -11062,6 +11867,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -11129,6 +11939,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T163" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -11196,6 +12011,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T164" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -11263,6 +12083,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T165" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -11330,6 +12155,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T166" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -11397,6 +12227,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T167" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -11492,6 +12327,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T168" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -11559,6 +12399,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T169" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -11626,6 +12471,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T170" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -11693,9 +12543,14 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T171" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S171"/>
+  <autoFilter ref="A1:T171"/>
 </worksheet>
 </file>
 
@@ -11798,6 +12653,11 @@
           <t xml:space="preserve">Annotated-correlation</t>
         </is>
       </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OncomiR/TS miRNA</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -11865,6 +12725,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -11932,6 +12797,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -11999,6 +12869,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -12066,6 +12941,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -12133,6 +13013,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -12200,6 +13085,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -12267,6 +13157,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -12334,6 +13229,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -12401,6 +13301,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -12468,6 +13373,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -12535,6 +13445,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -12602,6 +13517,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -12669,6 +13589,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -12736,6 +13661,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -12803,6 +13733,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -12870,6 +13805,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -12937,6 +13877,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -13004,6 +13949,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -13071,6 +14021,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -13138,6 +14093,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -13205,6 +14165,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -13272,6 +14237,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -13339,6 +14309,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -13406,6 +14381,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -13473,6 +14453,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -13540,6 +14525,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -13607,6 +14597,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -13674,6 +14669,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -13741,6 +14741,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -13808,6 +14813,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -13875,6 +14885,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -13942,6 +14957,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -14009,6 +15029,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -14076,6 +15101,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -14143,6 +15173,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -14210,6 +15245,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -14277,6 +15317,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tumor suppressor</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -14344,6 +15389,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -14411,6 +15461,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -14478,6 +15533,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -14545,6 +15605,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -14612,6 +15677,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -14679,6 +15749,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -14746,6 +15821,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OncomiR</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -14813,6 +15893,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -14908,6 +15993,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -15003,6 +16093,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -15098,6 +16193,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -15193,6 +16293,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -15260,6 +16365,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tumor suppressor</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -15327,6 +16437,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -15394,6 +16509,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -15461,6 +16581,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -15556,6 +16681,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -15651,6 +16781,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -15746,6 +16881,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -15813,6 +16953,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -15908,6 +17053,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -16003,6 +17153,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -16070,6 +17225,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -16137,6 +17297,11 @@
           <t xml:space="preserve">No</t>
         </is>
       </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -16204,6 +17369,11 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -16271,8 +17441,13 @@
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S64"/>
+  <autoFilter ref="A1:T64"/>
 </worksheet>
 </file>
</xml_diff>